<commit_message>
Migrate to SDL, update TODO
</commit_message>
<xml_diff>
--- a/TODO.xlsx
+++ b/TODO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trist\source\repos\sfml3D\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C431FD35-3A81-4041-84CA-7FEFDA9A6057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D21AB4-7B2A-4E3E-AF3C-C1F981CF48E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,36 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>PRIORITY</t>
   </si>
   <si>
-    <t>/*MAKE INTERACTING WITH VERTICES MORE INTUITIVE, MOVE TYPE DEFENITIONS OUTSIDE OF MESH FOR CONSISTENCY*/</t>
+    <t>ADD BUFFER FOR PIXELS(DON’T DRAW EACH INDIVIDUAL PIXEL AT THE START)</t>
   </si>
   <si>
-    <t>FINISH CAMERA ROTATION</t>
+    <t>ADD Z DEPTH BUFFER</t>
   </si>
   <si>
-    <t>ADD LIGHTING OBJECTS</t>
-  </si>
-  <si>
-    <t>TEXTURING</t>
-  </si>
-  <si>
-    <t>COLLISION</t>
-  </si>
-  <si>
-    <t>ANIMATION</t>
-  </si>
-  <si>
-    <t>/*TODO MODIFY VERTEX DATA TO ARRAY OF SIZE 3 (OPTIMIZE AS CURRENT ARCHITECTURE(AND MANY 3D RENDERERS) ONLY SUPPORTS MODELS MADE UP OF TRIANGLES ANYWAY)*/</t>
-  </si>
-  <si>
-    <t>FIX DEPTH ALGORITHM</t>
-  </si>
-  <si>
-    <t>ELAPSED TIME</t>
+    <t>ADD COLOR INTERPOLATION BETWEEN PIXELS</t>
   </si>
 </sst>
 </file>
@@ -382,7 +364,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -394,69 +376,50 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>